<commit_message>
Cau hinh toan bo he thong
</commit_message>
<xml_diff>
--- a/Danh_Sach_San_Pham_Cova.xlsx
+++ b/Danh_Sach_San_Pham_Cova.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:M34"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
     <col min="2" max="2" width="45.83203125" customWidth="1"/>
@@ -407,6 +407,11 @@
     <col min="6" max="6" width="15.83203125" customWidth="1"/>
     <col min="7" max="7" width="15.83203125" customWidth="1"/>
     <col min="8" max="8" width="15.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" customWidth="1"/>
+    <col min="11" max="11" width="12.83203125" customWidth="1"/>
+    <col min="12" max="12" width="12.83203125" customWidth="1"/>
+    <col min="13" max="13" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -434,6 +439,21 @@
       <c r="H1" t="str">
         <v>Giá Túi</v>
       </c>
+      <c r="I1" t="str">
+        <v>KL Thùng</v>
+      </c>
+      <c r="J1" t="str">
+        <v>KL Lon</v>
+      </c>
+      <c r="K1" t="str">
+        <v>KL Hộp</v>
+      </c>
+      <c r="L1" t="str">
+        <v>KL Bao</v>
+      </c>
+      <c r="M1" t="str">
+        <v>KL Túi</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -460,6 +480,21 @@
       <c r="H2">
         <v>0</v>
       </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -486,6 +521,21 @@
       <c r="H3">
         <v>0</v>
       </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v/>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -512,6 +562,21 @@
       <c r="H4">
         <v>125000</v>
       </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -538,6 +603,21 @@
       <c r="H5">
         <v>0</v>
       </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v>1.0kg</v>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -564,6 +644,21 @@
       <c r="H6">
         <v>0</v>
       </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
+        <v>4.5kg</v>
+      </c>
+      <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -590,6 +685,21 @@
       <c r="H7">
         <v>0</v>
       </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v>4.5kg</v>
+      </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="str">
+        <v>10.5kg</v>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -616,6 +726,21 @@
       <c r="H8">
         <v>0</v>
       </c>
+      <c r="I8" t="str">
+        <v>19kg</v>
+      </c>
+      <c r="J8" t="str">
+        <v>4.5kg</v>
+      </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -642,6 +767,21 @@
       <c r="H9">
         <v>0</v>
       </c>
+      <c r="I9" t="str">
+        <v>19kg</v>
+      </c>
+      <c r="J9" t="str">
+        <v>4.5kg</v>
+      </c>
+      <c r="K9" t="str">
+        <v/>
+      </c>
+      <c r="L9" t="str">
+        <v/>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -668,6 +808,21 @@
       <c r="H10">
         <v>0</v>
       </c>
+      <c r="I10" t="str">
+        <v>20.5kg</v>
+      </c>
+      <c r="J10" t="str">
+        <v>5.5kg</v>
+      </c>
+      <c r="K10" t="str">
+        <v/>
+      </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
+      <c r="M10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -694,6 +849,21 @@
       <c r="H11">
         <v>0</v>
       </c>
+      <c r="I11" t="str">
+        <v>19.5kg</v>
+      </c>
+      <c r="J11" t="str">
+        <v>5.5kg</v>
+      </c>
+      <c r="K11" t="str">
+        <v/>
+      </c>
+      <c r="L11" t="str">
+        <v/>
+      </c>
+      <c r="M11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -720,6 +890,21 @@
       <c r="H12">
         <v>0</v>
       </c>
+      <c r="I12" t="str">
+        <v>19kg</v>
+      </c>
+      <c r="J12" t="str">
+        <v>5.3kg</v>
+      </c>
+      <c r="K12" t="str">
+        <v>1.2kg</v>
+      </c>
+      <c r="L12" t="str">
+        <v/>
+      </c>
+      <c r="M12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -746,6 +931,21 @@
       <c r="H13">
         <v>0</v>
       </c>
+      <c r="I13" t="str">
+        <v>19kg</v>
+      </c>
+      <c r="J13" t="str">
+        <v>5.3kg</v>
+      </c>
+      <c r="K13" t="str">
+        <v>1.2kg</v>
+      </c>
+      <c r="L13" t="str">
+        <v/>
+      </c>
+      <c r="M13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -772,6 +972,21 @@
       <c r="H14">
         <v>0</v>
       </c>
+      <c r="I14" t="str">
+        <v>23.5kg</v>
+      </c>
+      <c r="J14" t="str">
+        <v>7.0kg</v>
+      </c>
+      <c r="K14" t="str">
+        <v/>
+      </c>
+      <c r="L14" t="str">
+        <v/>
+      </c>
+      <c r="M14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -798,6 +1013,21 @@
       <c r="H15">
         <v>0</v>
       </c>
+      <c r="I15" t="str">
+        <v>22.5kg</v>
+      </c>
+      <c r="J15" t="str">
+        <v>6.3kg</v>
+      </c>
+      <c r="K15" t="str">
+        <v/>
+      </c>
+      <c r="L15" t="str">
+        <v/>
+      </c>
+      <c r="M15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -824,6 +1054,21 @@
       <c r="H16">
         <v>0</v>
       </c>
+      <c r="I16" t="str">
+        <v>22.5kg</v>
+      </c>
+      <c r="J16" t="str">
+        <v>6.3kg</v>
+      </c>
+      <c r="K16" t="str">
+        <v/>
+      </c>
+      <c r="L16" t="str">
+        <v/>
+      </c>
+      <c r="M16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -850,6 +1095,21 @@
       <c r="H17">
         <v>0</v>
       </c>
+      <c r="I17" t="str">
+        <v>22.5kg</v>
+      </c>
+      <c r="J17" t="str">
+        <v>6.3kg</v>
+      </c>
+      <c r="K17" t="str">
+        <v/>
+      </c>
+      <c r="L17" t="str">
+        <v/>
+      </c>
+      <c r="M17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -876,6 +1136,21 @@
       <c r="H18">
         <v>0</v>
       </c>
+      <c r="I18" t="str">
+        <v>23.5kg</v>
+      </c>
+      <c r="J18" t="str">
+        <v>7.0kg</v>
+      </c>
+      <c r="K18" t="str">
+        <v/>
+      </c>
+      <c r="L18" t="str">
+        <v/>
+      </c>
+      <c r="M18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -902,6 +1177,21 @@
       <c r="H19">
         <v>0</v>
       </c>
+      <c r="I19" t="str">
+        <v>22.0kg</v>
+      </c>
+      <c r="J19" t="str">
+        <v>6.0kg</v>
+      </c>
+      <c r="K19" t="str">
+        <v/>
+      </c>
+      <c r="L19" t="str">
+        <v/>
+      </c>
+      <c r="M19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -928,6 +1218,21 @@
       <c r="H20">
         <v>0</v>
       </c>
+      <c r="I20" t="str">
+        <v>22.0kg</v>
+      </c>
+      <c r="J20" t="str">
+        <v>6.0kg</v>
+      </c>
+      <c r="K20" t="str">
+        <v/>
+      </c>
+      <c r="L20" t="str">
+        <v/>
+      </c>
+      <c r="M20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -954,6 +1259,21 @@
       <c r="H21">
         <v>0</v>
       </c>
+      <c r="I21" t="str">
+        <v>23.5kg</v>
+      </c>
+      <c r="J21" t="str">
+        <v>7kg</v>
+      </c>
+      <c r="K21" t="str">
+        <v/>
+      </c>
+      <c r="L21" t="str">
+        <v/>
+      </c>
+      <c r="M21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -980,6 +1300,21 @@
       <c r="H22">
         <v>0</v>
       </c>
+      <c r="I22" t="str">
+        <v>23.5kg</v>
+      </c>
+      <c r="J22" t="str">
+        <v>7.0kg</v>
+      </c>
+      <c r="K22" t="str">
+        <v/>
+      </c>
+      <c r="L22" t="str">
+        <v/>
+      </c>
+      <c r="M22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -1006,6 +1341,21 @@
       <c r="H23">
         <v>0</v>
       </c>
+      <c r="I23" t="str">
+        <v>19.0kg</v>
+      </c>
+      <c r="J23" t="str">
+        <v>5.5kg</v>
+      </c>
+      <c r="K23" t="str">
+        <v/>
+      </c>
+      <c r="L23" t="str">
+        <v/>
+      </c>
+      <c r="M23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -1032,6 +1382,21 @@
       <c r="H24">
         <v>0</v>
       </c>
+      <c r="I24" t="str">
+        <v>19.0kg</v>
+      </c>
+      <c r="J24" t="str">
+        <v>5.5kg</v>
+      </c>
+      <c r="K24" t="str">
+        <v/>
+      </c>
+      <c r="L24" t="str">
+        <v/>
+      </c>
+      <c r="M24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -1058,6 +1423,21 @@
       <c r="H25">
         <v>0</v>
       </c>
+      <c r="I25" t="str">
+        <v>19.0kg</v>
+      </c>
+      <c r="J25" t="str">
+        <v>5.5kg</v>
+      </c>
+      <c r="K25" t="str">
+        <v/>
+      </c>
+      <c r="L25" t="str">
+        <v/>
+      </c>
+      <c r="M25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -1084,6 +1464,21 @@
       <c r="H26">
         <v>0</v>
       </c>
+      <c r="I26" t="str">
+        <v>19.0kg</v>
+      </c>
+      <c r="J26" t="str">
+        <v>5.5kg</v>
+      </c>
+      <c r="K26" t="str">
+        <v/>
+      </c>
+      <c r="L26" t="str">
+        <v/>
+      </c>
+      <c r="M26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -1110,6 +1505,21 @@
       <c r="H27">
         <v>0</v>
       </c>
+      <c r="I27" t="str">
+        <v>23.0kg</v>
+      </c>
+      <c r="J27" t="str">
+        <v>6.5kg</v>
+      </c>
+      <c r="K27" t="str">
+        <v/>
+      </c>
+      <c r="L27" t="str">
+        <v/>
+      </c>
+      <c r="M27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -1136,6 +1546,21 @@
       <c r="H28">
         <v>0</v>
       </c>
+      <c r="I28" t="str">
+        <v>23.0kg</v>
+      </c>
+      <c r="J28" t="str">
+        <v>6.5kg</v>
+      </c>
+      <c r="K28" t="str">
+        <v/>
+      </c>
+      <c r="L28" t="str">
+        <v/>
+      </c>
+      <c r="M28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -1162,6 +1587,21 @@
       <c r="H29">
         <v>0</v>
       </c>
+      <c r="I29" t="str">
+        <v>23.5kg</v>
+      </c>
+      <c r="J29" t="str">
+        <v>7.0kg</v>
+      </c>
+      <c r="K29" t="str">
+        <v/>
+      </c>
+      <c r="L29" t="str">
+        <v/>
+      </c>
+      <c r="M29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -1188,6 +1628,21 @@
       <c r="H30">
         <v>0</v>
       </c>
+      <c r="I30" t="str">
+        <v>22.5kg</v>
+      </c>
+      <c r="J30" t="str">
+        <v>6.0kg</v>
+      </c>
+      <c r="K30" t="str">
+        <v/>
+      </c>
+      <c r="L30" t="str">
+        <v/>
+      </c>
+      <c r="M30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -1214,6 +1669,21 @@
       <c r="H31">
         <v>0</v>
       </c>
+      <c r="I31" t="str">
+        <v>19.5kg</v>
+      </c>
+      <c r="J31" t="str">
+        <v>5.5kg</v>
+      </c>
+      <c r="K31" t="str">
+        <v/>
+      </c>
+      <c r="L31" t="str">
+        <v/>
+      </c>
+      <c r="M31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -1240,6 +1710,21 @@
       <c r="H32">
         <v>0</v>
       </c>
+      <c r="I32" t="str">
+        <v>19.0kg</v>
+      </c>
+      <c r="J32" t="str">
+        <v>5.3kg</v>
+      </c>
+      <c r="K32" t="str">
+        <v/>
+      </c>
+      <c r="L32" t="str">
+        <v/>
+      </c>
+      <c r="M32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -1266,6 +1751,21 @@
       <c r="H33">
         <v>0</v>
       </c>
+      <c r="I33" t="str">
+        <v>19.0kg</v>
+      </c>
+      <c r="J33" t="str">
+        <v>5.3kg</v>
+      </c>
+      <c r="K33" t="str">
+        <v>1.2kg</v>
+      </c>
+      <c r="L33" t="str">
+        <v/>
+      </c>
+      <c r="M33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -1292,10 +1792,25 @@
       <c r="H34">
         <v>0</v>
       </c>
+      <c r="I34" t="str">
+        <v>19.0kg</v>
+      </c>
+      <c r="J34" t="str">
+        <v>5.5kg</v>
+      </c>
+      <c r="K34" t="str">
+        <v>1.2kg</v>
+      </c>
+      <c r="L34" t="str">
+        <v/>
+      </c>
+      <c r="M34" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H34"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M34"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>